<commit_message>
Daily recap, matchup updates, learning and research 2026-08-27
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-27.xlsx
+++ b/data/k-props/2026-08-27.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="73">
   <si>
     <t>date</t>
   </si>
@@ -160,6 +160,9 @@
     <t>Baltimore Orioles @ St. Louis Cardinals</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>Gordon Graceffo</t>
   </si>
   <si>
@@ -175,6 +178,9 @@
     <t>Gerrit Cole</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
     <t>6-7</t>
   </si>
   <si>
@@ -208,6 +214,9 @@
     <t>Chris Sale</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>Jose Cabrera</t>
   </si>
   <si>
@@ -215,6 +224,9 @@
   </si>
   <si>
     <t>Limited starter</t>
+  </si>
+  <si>
+    <t>W</t>
   </si>
   <si>
     <t>Landen Roupp</t>
@@ -983,8 +995,14 @@
       <c r="Y4">
         <v>0.9253</v>
       </c>
+      <c r="Z4">
+        <v>7</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>49</v>
+      </c>
+      <c r="AB4">
+        <v>-0.03</v>
       </c>
       <c r="AC4" t="s">
         <v>44</v>
@@ -1003,6 +1021,18 @@
       </c>
       <c r="AH4">
         <v>0.22</v>
+      </c>
+      <c r="AI4">
+        <v>2.75</v>
+      </c>
+      <c r="AJ4">
+        <v>2.75</v>
+      </c>
+      <c r="AK4">
+        <v>2.53</v>
+      </c>
+      <c r="AL4">
+        <v>2.53</v>
       </c>
       <c r="AM4">
         <v>4.47</v>
@@ -1013,7 +1043,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
         <v>48</v>
@@ -1022,7 +1052,7 @@
         <v>823014</v>
       </c>
       <c r="H5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I5">
         <v>3</v>
@@ -1105,7 +1135,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C6">
         <v>4.5</v>
@@ -1117,7 +1147,7 @@
         <v>-170</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G6">
         <v>823503</v>
@@ -1176,8 +1206,14 @@
       <c r="Y6">
         <v>0.953</v>
       </c>
+      <c r="Z6">
+        <v>6</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>49</v>
+      </c>
+      <c r="AB6">
+        <v>0.44</v>
       </c>
       <c r="AC6" t="s">
         <v>44</v>
@@ -1196,6 +1232,18 @@
       </c>
       <c r="AH6">
         <v>0.22</v>
+      </c>
+      <c r="AI6">
+        <v>1.28</v>
+      </c>
+      <c r="AJ6">
+        <v>1.28</v>
+      </c>
+      <c r="AK6">
+        <v>1.06</v>
+      </c>
+      <c r="AL6">
+        <v>1.06</v>
       </c>
       <c r="AM6">
         <v>4.94</v>
@@ -1206,7 +1254,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C7">
         <v>5.5</v>
@@ -1218,7 +1266,7 @@
         <v>-113</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G7">
         <v>823503</v>
@@ -1277,8 +1325,14 @@
       <c r="Y7">
         <v>0.9915</v>
       </c>
+      <c r="Z7">
+        <v>5</v>
+      </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>55</v>
+      </c>
+      <c r="AB7">
+        <v>0.24</v>
       </c>
       <c r="AC7" t="s">
         <v>44</v>
@@ -1287,7 +1341,7 @@
         <v>6.31</v>
       </c>
       <c r="AE7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AF7">
         <v>0.2716</v>
@@ -1297,6 +1351,18 @@
       </c>
       <c r="AH7">
         <v>-0.57</v>
+      </c>
+      <c r="AI7">
+        <v>-1.31</v>
+      </c>
+      <c r="AJ7">
+        <v>1.31</v>
+      </c>
+      <c r="AK7">
+        <v>-0.74</v>
+      </c>
+      <c r="AL7">
+        <v>0.74</v>
       </c>
       <c r="AM7">
         <v>5.74</v>
@@ -1307,7 +1373,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C8">
         <v>4.5</v>
@@ -1319,7 +1385,7 @@
         <v>105</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G8">
         <v>822771</v>
@@ -1378,8 +1444,14 @@
       <c r="Y8">
         <v>0.9309</v>
       </c>
+      <c r="Z8">
+        <v>3</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>55</v>
+      </c>
+      <c r="AB8">
+        <v>-0.34</v>
       </c>
       <c r="AC8" t="s">
         <v>44</v>
@@ -1398,6 +1470,18 @@
       </c>
       <c r="AH8">
         <v>0.22</v>
+      </c>
+      <c r="AI8">
+        <v>-0.94</v>
+      </c>
+      <c r="AJ8">
+        <v>0.94</v>
+      </c>
+      <c r="AK8">
+        <v>-1.16</v>
+      </c>
+      <c r="AL8">
+        <v>1.16</v>
       </c>
       <c r="AM8">
         <v>4.16</v>
@@ -1408,10 +1492,10 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G9">
         <v>822771</v>
@@ -1500,7 +1584,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C10">
         <v>8.5</v>
@@ -1512,7 +1596,7 @@
         <v>-109</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G10">
         <v>823581</v>
@@ -1571,8 +1655,14 @@
       <c r="Y10">
         <v>1.0166</v>
       </c>
+      <c r="Z10">
+        <v>6</v>
+      </c>
       <c r="AA10" t="s">
-        <v>44</v>
+        <v>55</v>
+      </c>
+      <c r="AB10">
+        <v>0.39</v>
       </c>
       <c r="AC10" t="s">
         <v>44</v>
@@ -1581,7 +1671,7 @@
         <v>9.96</v>
       </c>
       <c r="AE10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AF10">
         <v>0.3908</v>
@@ -1591,6 +1681,18 @@
       </c>
       <c r="AH10">
         <v>-1.07</v>
+      </c>
+      <c r="AI10">
+        <v>-3.96</v>
+      </c>
+      <c r="AJ10">
+        <v>3.96</v>
+      </c>
+      <c r="AK10">
+        <v>-2.89</v>
+      </c>
+      <c r="AL10">
+        <v>2.89</v>
       </c>
       <c r="AM10">
         <v>8.89</v>
@@ -1601,7 +1703,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C11">
         <v>4.5</v>
@@ -1613,7 +1715,7 @@
         <v>126</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G11">
         <v>823581</v>
@@ -1672,8 +1774,14 @@
       <c r="Y11">
         <v>0.88</v>
       </c>
+      <c r="Z11">
+        <v>3</v>
+      </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>55</v>
+      </c>
+      <c r="AB11">
+        <v>0.45</v>
       </c>
       <c r="AC11" t="s">
         <v>44</v>
@@ -1692,6 +1800,18 @@
       </c>
       <c r="AH11">
         <v>0.22</v>
+      </c>
+      <c r="AI11">
+        <v>-1.73</v>
+      </c>
+      <c r="AJ11">
+        <v>1.73</v>
+      </c>
+      <c r="AK11">
+        <v>-1.95</v>
+      </c>
+      <c r="AL11">
+        <v>1.95</v>
       </c>
       <c r="AM11">
         <v>4.95</v>
@@ -1702,7 +1822,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C12">
         <v>5.5</v>
@@ -1714,7 +1834,7 @@
         <v>126</v>
       </c>
       <c r="F12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G12">
         <v>824879</v>
@@ -1773,8 +1893,14 @@
       <c r="Y12">
         <v>0.9917</v>
       </c>
+      <c r="Z12">
+        <v>8</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>49</v>
+      </c>
+      <c r="AB12">
+        <v>0.44</v>
       </c>
       <c r="AC12" t="s">
         <v>44</v>
@@ -1783,7 +1909,7 @@
         <v>6.51</v>
       </c>
       <c r="AE12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AF12">
         <v>0.2492</v>
@@ -1793,6 +1919,18 @@
       </c>
       <c r="AH12">
         <v>-0.57</v>
+      </c>
+      <c r="AI12">
+        <v>1.49</v>
+      </c>
+      <c r="AJ12">
+        <v>1.49</v>
+      </c>
+      <c r="AK12">
+        <v>2.06</v>
+      </c>
+      <c r="AL12">
+        <v>2.06</v>
       </c>
       <c r="AM12">
         <v>5.94</v>
@@ -1803,7 +1941,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C13">
         <v>7.5</v>
@@ -1815,7 +1953,7 @@
         <v>-151</v>
       </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G13">
         <v>824879</v>
@@ -1874,17 +2012,23 @@
       <c r="Y13">
         <v>0.9741</v>
       </c>
+      <c r="Z13">
+        <v>11</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>49</v>
+      </c>
+      <c r="AB13">
+        <v>-1.08</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="AD13">
         <v>7.49</v>
       </c>
       <c r="AE13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AF13">
         <v>0.3299</v>
@@ -1894,6 +2038,18 @@
       </c>
       <c r="AH13">
         <v>-1.07</v>
+      </c>
+      <c r="AI13">
+        <v>3.51</v>
+      </c>
+      <c r="AJ13">
+        <v>3.51</v>
+      </c>
+      <c r="AK13">
+        <v>4.58</v>
+      </c>
+      <c r="AL13">
+        <v>4.58</v>
       </c>
       <c r="AM13">
         <v>6.42</v>
@@ -1904,7 +2060,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C14">
         <v>3.5</v>
@@ -1916,13 +2072,13 @@
         <v>-113</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G14">
         <v>823179</v>
       </c>
       <c r="H14" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I14">
         <v>4.4</v>
@@ -1975,11 +2131,17 @@
       <c r="Y14">
         <v>1.0025</v>
       </c>
+      <c r="Z14">
+        <v>4</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>49</v>
+      </c>
+      <c r="AB14">
+        <v>0.75</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="AD14">
         <v>4.03</v>
@@ -1995,6 +2157,18 @@
       </c>
       <c r="AH14">
         <v>0.22</v>
+      </c>
+      <c r="AI14">
+        <v>-0.03</v>
+      </c>
+      <c r="AJ14">
+        <v>0.03</v>
+      </c>
+      <c r="AK14">
+        <v>-0.25</v>
+      </c>
+      <c r="AL14">
+        <v>0.25</v>
       </c>
       <c r="AM14">
         <v>4.25</v>
@@ -2005,7 +2179,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2017,7 +2191,7 @@
         <v>-122</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G15">
         <v>823179</v>
@@ -2076,11 +2250,17 @@
       <c r="Y15">
         <v>0.88</v>
       </c>
+      <c r="Z15">
+        <v>3</v>
+      </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>55</v>
+      </c>
+      <c r="AB15">
+        <v>-0.9</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="AD15">
         <v>3.38</v>
@@ -2096,6 +2276,18 @@
       </c>
       <c r="AH15">
         <v>0.22</v>
+      </c>
+      <c r="AI15">
+        <v>-0.38</v>
+      </c>
+      <c r="AJ15">
+        <v>0.38</v>
+      </c>
+      <c r="AK15">
+        <v>-0.6</v>
+      </c>
+      <c r="AL15">
+        <v>0.6</v>
       </c>
       <c r="AM15">
         <v>3.6</v>

</xml_diff>